<commit_message>
unit and structure preliminary content
</commit_message>
<xml_diff>
--- a/Assets/Data/Data.xlsx
+++ b/Assets/Data/Data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="84">
   <si>
     <t xml:space="preserve">Num Code</t>
   </si>
@@ -70,6 +70,9 @@
     <t xml:space="preserve">garrison</t>
   </si>
   <si>
+    <t xml:space="preserve">notes</t>
+  </si>
+  <si>
     <t xml:space="preserve">structure</t>
   </si>
   <si>
@@ -85,7 +88,7 @@
     <t xml:space="preserve">knight</t>
   </si>
   <si>
-    <t xml:space="preserve">lechery</t>
+    <t xml:space="preserve">flechery</t>
   </si>
   <si>
     <t xml:space="preserve">archer</t>
@@ -124,178 +127,154 @@
     <t xml:space="preserve">god-maker</t>
   </si>
   <si>
+    <t xml:space="preserve">god</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gunsmith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gunner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peasant-homes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peasantry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peasant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mage-tower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-nest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dragon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">egg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-hatchery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gem-mine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-rider-roost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uncommon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-rider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">farm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pop-growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold-mine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold-income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">granary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">treasury</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunters-lodge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">this is a long sentence. I am testing if this breaks. We will see</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trading-post</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mage-academy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bigger-mage-tower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">archmage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">crystal-refinery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mage-university</t>
+  </si>
+  <si>
+    <t xml:space="preserve">work-house</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peasant-lodge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Health</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attack Speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attack Range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Move Speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description of the unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notes about the unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unit</t>
+  </si>
+  <si>
     <t xml:space="preserve">debug tool</t>
   </si>
   <si>
-    <t xml:space="preserve">god</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gunsmith</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gunner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peasant-homes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peasantry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">peasant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mage-tower</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-nest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">makes dragon eggs. Basic dragon structure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dragon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">egg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-hatchery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gem-mine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">basic resource structure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-rider-roost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uncommon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-rider</t>
-  </si>
-  <si>
-    <t xml:space="preserve">farm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pop-growth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold-mine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold-income</t>
-  </si>
-  <si>
-    <t xml:space="preserve">granary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">advanced resource structure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">treasury</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold income is not currently implemented. We should uh, do that.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hunters-lodge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">weak but plentiful ranged units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">could give pop growth + hunters as a unique thing, since they hunt + fight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hunters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rare resource structure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">trading post</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mage-academy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">advanced mage producer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bigger-mage-tower</t>
-  </si>
-  <si>
-    <t xml:space="preserve">archmage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">crystal refinery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mage-university</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rare mage producer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Health</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attack Speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attack Range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Move Speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description of the unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notes about the unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hunter</t>
-  </si>
-  <si>
     <t xml:space="preserve">gold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resource.png</t>
   </si>
 </sst>
 </file>
@@ -968,11 +947,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultColWidth="8.75390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.14"/>
@@ -1036,34 +1015,38 @@
       <c r="B2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
+      <c r="C2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>2</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N2" s="10" t="n">
         <v>4</v>
@@ -1074,36 +1057,40 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+        <v>21</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H3" s="8" t="n">
         <v>3</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J3" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N3" s="10" t="n">
         <v>4</v>
@@ -1114,36 +1101,40 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
+        <v>23</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>2</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N4" s="10" t="n">
         <v>4</v>
@@ -1154,36 +1145,40 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+        <v>25</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>2</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N5" s="10" t="n">
         <v>4</v>
@@ -1194,76 +1189,84 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>6</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N6" s="10" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+        <v>29</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H7" s="8" t="n">
         <v>4</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N7" s="10" t="n">
         <v>2</v>
@@ -1274,36 +1277,40 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
+        <v>31</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E8" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N8" s="10" t="n">
         <v>4</v>
@@ -1314,34 +1321,34 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>2</v>
@@ -1360,28 +1367,32 @@
       <c r="B10" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="C10" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E10" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H10" s="8" t="n">
         <v>7</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>2</v>
@@ -1393,35 +1404,39 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
+      <c r="C11" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>2</v>
@@ -1430,7 +1445,7 @@
         <v>39</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1440,31 +1455,35 @@
       <c r="B12" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
+      <c r="C12" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E12" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H12" s="8" t="n">
         <v>5</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>43</v>
@@ -1481,17 +1500,19 @@
         <v>44</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="7"/>
-      <c r="E13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="G13" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H13" s="8" t="n">
         <v>2</v>
@@ -1503,53 +1524,57 @@
         <v>3</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N13" s="10" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
+        <v>47</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E14" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H14" s="8" t="n">
         <v>10</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N14" s="10" t="n">
         <v>1</v>
@@ -1560,32 +1585,34 @@
         <v>15</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E15" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H15" s="8" t="n">
         <v>5</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J15" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0</v>
@@ -1594,7 +1621,7 @@
         <v>42</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,36 +1629,40 @@
         <v>16</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="L16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="H16" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="J16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M16" s="7" t="s">
-        <v>54</v>
       </c>
       <c r="N16" s="10" t="n">
         <v>1</v>
@@ -1642,38 +1673,40 @@
         <v>17</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E17" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J17" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>0</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="N17" s="10" t="n">
         <v>1</v>
@@ -1684,38 +1717,40 @@
         <v>18</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E18" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J18" s="8" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L18" s="8" t="n">
         <v>0</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N18" s="10" t="n">
         <v>1</v>
@@ -1726,26 +1761,28 @@
         <v>19</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E19" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J19" s="8" t="n">
         <v>1</v>
@@ -1757,39 +1794,39 @@
         <v>2</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="N19" s="10" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="n">
         <v>20</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H20" s="8" t="n">
         <v>4</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J20" s="8" t="n">
         <v>1</v>
@@ -1801,10 +1838,10 @@
         <v>2</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N20" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1812,40 +1849,40 @@
         <v>21</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H21" s="8" t="n">
         <v>1</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J21" s="8" t="n">
         <v>5</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L21" s="8" t="n">
         <v>0</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="N21" s="10" t="n">
         <v>10</v>
@@ -1856,26 +1893,28 @@
         <v>22</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E22" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>1</v>
@@ -1887,10 +1926,10 @@
         <v>3</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="N22" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,26 +1937,28 @@
         <v>23</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D23" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E23" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J23" s="8" t="n">
         <v>1</v>
@@ -1929,10 +1970,10 @@
         <v>3</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="N23" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1940,20 +1981,22 @@
         <v>24</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D24" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E24" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>41</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H24" s="8" t="n">
         <v>6</v>
@@ -1965,7 +2008,7 @@
         <v>3</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L24" s="8" t="n">
         <v>3</v>
@@ -1982,18 +2025,22 @@
         <v>25</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
+        <v>66</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E25" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>41</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>6</v>
@@ -2005,13 +2052,13 @@
         <v>1</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L25" s="8" t="n">
         <v>1</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="N25" s="10" t="n">
         <v>1</v>
@@ -2022,62 +2069,66 @@
         <v>26</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D26" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E26" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>41</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L26" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>42</v>
       </c>
       <c r="N26" s="10" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="n">
         <v>27</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="E27" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>41</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="H27" s="8" t="n">
         <v>10</v>
@@ -2089,21 +2140,109 @@
         <v>3</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L27" s="8" t="n">
         <v>3</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="N27" s="10" t="n">
         <v>3</v>
       </c>
     </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="J28" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="K28" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="L28" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="N28" s="10" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="I29" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="K29" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="L29" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="N29" s="10" t="n">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G27" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G29" type="list">
       <formula1>INDIRECT("RarityData")</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2162,25 +2301,25 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="M1" s="12" t="s">
         <v>78</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="M1" s="12" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2188,19 +2327,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="7" t="n">
@@ -2227,15 +2366,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+        <v>22</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E3" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="7" t="n">
@@ -2262,15 +2405,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
+        <v>24</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E4" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="7" t="n">
@@ -2297,15 +2444,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+        <v>26</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E5" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5" s="7" t="n">
@@ -2332,25 +2483,29 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
+        <v>28</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E6" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>0.5</v>
@@ -2367,15 +2522,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+        <v>30</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E7" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7" t="n">
@@ -2402,15 +2561,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
+        <v>32</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E8" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7" t="n">
@@ -2437,15 +2600,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+        <v>48</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E9" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7" t="n">
@@ -2474,13 +2641,17 @@
       <c r="B10" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="C10" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E10" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="7" t="n">
@@ -2509,10 +2680,14 @@
       <c r="B11" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
+      <c r="C11" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E11" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>38</v>
@@ -2545,16 +2720,16 @@
         <v>34</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" s="7" t="n">
@@ -2581,15 +2756,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
+        <v>52</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E13" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7" t="n">
@@ -2618,10 +2797,14 @@
       <c r="B14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
+      <c r="C14" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E14" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>41</v>
@@ -2637,7 +2820,7 @@
         <v>15</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="7" t="n">
         <v>3</v>
@@ -2651,12 +2834,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
+        <v>61</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E15" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>38</v>
@@ -2683,15 +2870,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
+        <v>67</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="E16" s="7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>41</v>
@@ -2707,7 +2898,7 @@
         <v>30</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L16" s="7" t="n">
         <v>4</v>
@@ -2758,34 +2949,34 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>90</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>90</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2793,15 +2984,15 @@
         <v>42</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>90</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>90</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2836,17 +3027,17 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
basic implementation of spire regen, and default resource leveling
</commit_message>
<xml_diff>
--- a/Assets/Data/Data.xlsx
+++ b/Assets/Data/Data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" state="visible" r:id="rId3"/>
@@ -175,6 +175,9 @@
     <t xml:space="preserve">gem-mine</t>
   </si>
   <si>
+    <t xml:space="preserve">gem-income</t>
+  </si>
+  <si>
     <t xml:space="preserve">dragon-rider-roost</t>
   </si>
   <si>
@@ -193,33 +196,33 @@
     <t xml:space="preserve">gold-mine</t>
   </si>
   <si>
-    <t xml:space="preserve">gold-income</t>
+    <t xml:space="preserve">gold</t>
   </si>
   <si>
     <t xml:space="preserve">granary</t>
   </si>
   <si>
+    <t xml:space="preserve">trading-post</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunters-lodge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">this is a long sentence. I am testing if this breaks. We will see</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rare</t>
+  </si>
+  <si>
     <t xml:space="preserve">treasury</t>
   </si>
   <si>
-    <t xml:space="preserve">hunters-lodge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">this is a long sentence. I am testing if this breaks. We will see</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hunter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">trading-post</t>
-  </si>
-  <si>
     <t xml:space="preserve">mage-academy</t>
   </si>
   <si>
@@ -272,9 +275,6 @@
   </si>
   <si>
     <t xml:space="preserve">debug tool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold</t>
   </si>
 </sst>
 </file>
@@ -1521,7 +1521,7 @@
         <v>42</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" s="9" t="s">
         <v>19</v>
@@ -1618,10 +1618,10 @@
         <v>0</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1629,7 +1629,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>2</v>
@@ -1644,7 +1644,7 @@
         <v>45</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H16" s="8" t="n">
         <v>15</v>
@@ -1662,7 +1662,7 @@
         <v>1</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N16" s="10" t="n">
         <v>1</v>
@@ -1673,7 +1673,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>2</v>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N17" s="10" t="n">
         <v>1</v>
@@ -1717,7 +1717,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>2</v>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N18" s="10" t="n">
         <v>1</v>
@@ -1761,7 +1761,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>2</v>
@@ -1776,7 +1776,7 @@
         <v>38</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>3</v>
@@ -1794,7 +1794,7 @@
         <v>2</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N19" s="10" t="n">
         <v>2</v>
@@ -1805,7 +1805,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>2</v>
@@ -1820,7 +1820,7 @@
         <v>38</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H20" s="8" t="n">
         <v>4</v>
@@ -1838,7 +1838,7 @@
         <v>2</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N20" s="10" t="n">
         <v>2</v>
@@ -1849,13 +1849,13 @@
         <v>21</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>2</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>16</v>
@@ -1882,7 +1882,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N21" s="10" t="n">
         <v>10</v>
@@ -1893,7 +1893,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>2</v>
@@ -1908,7 +1908,7 @@
         <v>38</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>7</v>
@@ -1926,7 +1926,7 @@
         <v>3</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N22" s="10" t="n">
         <v>3</v>
@@ -1937,7 +1937,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>2</v>
@@ -1952,7 +1952,7 @@
         <v>38</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H23" s="8" t="n">
         <v>8</v>
@@ -1970,7 +1970,7 @@
         <v>3</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N23" s="10" t="n">
         <v>3</v>
@@ -1981,7 +1981,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>2</v>
@@ -1996,7 +1996,7 @@
         <v>41</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H24" s="8" t="n">
         <v>6</v>
@@ -2025,7 +2025,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>2</v>
@@ -2040,16 +2040,16 @@
         <v>41</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I25" s="9" t="s">
         <v>42</v>
       </c>
       <c r="J25" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K25" s="9" t="s">
         <v>19</v>
@@ -2058,7 +2058,7 @@
         <v>1</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N25" s="10" t="n">
         <v>1</v>
@@ -2069,7 +2069,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>2</v>
@@ -2084,7 +2084,7 @@
         <v>41</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H26" s="8" t="n">
         <v>10</v>
@@ -2102,10 +2102,10 @@
         <v>0</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="N26" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2113,7 +2113,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>2</v>
@@ -2128,7 +2128,7 @@
         <v>41</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H27" s="8" t="n">
         <v>10</v>
@@ -2146,7 +2146,7 @@
         <v>3</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N27" s="10" t="n">
         <v>3</v>
@@ -2157,7 +2157,7 @@
         <v>28</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>2</v>
@@ -2172,7 +2172,7 @@
         <v>38</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H28" s="8" t="n">
         <v>3</v>
@@ -2201,7 +2201,7 @@
         <v>29</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>2</v>
@@ -2216,7 +2216,7 @@
         <v>38</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H29" s="8" t="n">
         <v>6</v>
@@ -2301,25 +2301,25 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2330,13 +2330,13 @@
         <v>20</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>17</v>
@@ -2369,13 +2369,13 @@
         <v>22</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>17</v>
@@ -2408,13 +2408,13 @@
         <v>24</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>17</v>
@@ -2447,13 +2447,13 @@
         <v>26</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>17</v>
@@ -2486,13 +2486,13 @@
         <v>28</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>17</v>
@@ -2525,13 +2525,13 @@
         <v>30</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>17</v>
@@ -2564,13 +2564,13 @@
         <v>32</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>17</v>
@@ -2603,13 +2603,13 @@
         <v>48</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>45</v>
@@ -2642,13 +2642,13 @@
         <v>36</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>17</v>
@@ -2681,13 +2681,13 @@
         <v>39</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>38</v>
@@ -2720,13 +2720,13 @@
         <v>34</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>81</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>17</v>
@@ -2756,16 +2756,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>45</v>
@@ -2798,13 +2798,13 @@
         <v>43</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>41</v>
@@ -2834,16 +2834,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>38</v>
@@ -2873,16 +2873,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>41</v>
@@ -2949,10 +2949,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2965,10 +2965,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2989,10 +2989,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -3032,12 +3032,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed peasants to be spawned based on city excess pop
</commit_message>
<xml_diff>
--- a/Assets/Data/Data.xlsx
+++ b/Assets/Data/Data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="82">
   <si>
     <t xml:space="preserve">Num Code</t>
   </si>
@@ -136,72 +136,75 @@
     <t xml:space="preserve">gunner</t>
   </si>
   <si>
-    <t xml:space="preserve">peasant-homes</t>
+    <t xml:space="preserve">gem-transmutator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gem-income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mage-tower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-nest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dragon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">egg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-hatchery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gem-mine</t>
   </si>
   <si>
     <t xml:space="preserve">Peasantry</t>
   </si>
   <si>
+    <t xml:space="preserve">dragon-rider-roost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uncommon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-rider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">farm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pop-growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold-mine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">granary</t>
+  </si>
+  <si>
     <t xml:space="preserve">peasant</t>
   </si>
   <si>
-    <t xml:space="preserve">mage-tower</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-nest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dragon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">egg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-hatchery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gem-mine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gem-income</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-rider-roost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uncommon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-rider</t>
-  </si>
-  <si>
-    <t xml:space="preserve">farm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pop-growth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold-mine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">granary</t>
-  </si>
-  <si>
     <t xml:space="preserve">trading-post</t>
   </si>
   <si>
@@ -217,9 +220,6 @@
     <t xml:space="preserve">mill</t>
   </si>
   <si>
-    <t xml:space="preserve">Rare</t>
-  </si>
-  <si>
     <t xml:space="preserve">treasury</t>
   </si>
   <si>
@@ -236,12 +236,6 @@
   </si>
   <si>
     <t xml:space="preserve">mage-university</t>
-  </si>
-  <si>
-    <t xml:space="preserve">work-house</t>
-  </si>
-  <si>
-    <t xml:space="preserve">peasant-lodge</t>
   </si>
   <si>
     <t xml:space="preserve">Structure</t>
@@ -947,7 +941,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultColWidth="8.75390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.51"/>
@@ -1037,7 +1031,7 @@
         <v>19</v>
       </c>
       <c r="J2" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>19</v>
@@ -1081,7 +1075,7 @@
         <v>19</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>19</v>
@@ -1125,7 +1119,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K4" s="9" t="s">
         <v>19</v>
@@ -1169,7 +1163,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K5" s="9" t="s">
         <v>19</v>
@@ -1257,7 +1251,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="9" t="s">
         <v>19</v>
@@ -1301,7 +1295,7 @@
         <v>19</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K8" s="9" t="s">
         <v>19</v>
@@ -1424,16 +1418,16 @@
         <v>38</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K11" s="9" t="s">
         <v>19</v>
@@ -1442,7 +1436,7 @@
         <v>2</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>5</v>
@@ -1453,7 +1447,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>2</v>
@@ -1465,7 +1459,7 @@
         <v>16</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>18</v>
@@ -1474,7 +1468,7 @@
         <v>5</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>2</v>
@@ -1486,7 +1480,7 @@
         <v>1</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N12" s="10" t="n">
         <v>1</v>
@@ -1497,7 +1491,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>2</v>
@@ -1509,7 +1503,7 @@
         <v>16</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>18</v>
@@ -1518,7 +1512,7 @@
         <v>2</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J13" s="8" t="n">
         <v>2</v>
@@ -1530,7 +1524,7 @@
         <v>1</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N13" s="10" t="n">
         <v>1</v>
@@ -1541,7 +1535,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>2</v>
@@ -1553,16 +1547,16 @@
         <v>16</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>18</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J14" s="8" t="n">
         <v>1</v>
@@ -1574,7 +1568,7 @@
         <v>1</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N14" s="10" t="n">
         <v>1</v>
@@ -1585,7 +1579,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>2</v>
@@ -1597,7 +1591,7 @@
         <v>16</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>18</v>
@@ -1618,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="N15" s="10" t="n">
         <v>1</v>
@@ -1629,7 +1623,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>2</v>
@@ -1641,16 +1635,16 @@
         <v>16</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J16" s="8" t="n">
         <v>1</v>
@@ -1662,7 +1656,7 @@
         <v>1</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N16" s="10" t="n">
         <v>1</v>
@@ -1673,7 +1667,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>2</v>
@@ -1685,7 +1679,7 @@
         <v>16</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>18</v>
@@ -1706,7 +1700,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N17" s="10" t="n">
         <v>1</v>
@@ -1717,7 +1711,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>2</v>
@@ -1729,7 +1723,7 @@
         <v>16</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>18</v>
@@ -1750,7 +1744,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="N18" s="10" t="n">
         <v>1</v>
@@ -1773,10 +1767,10 @@
         <v>16</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>3</v>
@@ -1788,13 +1782,13 @@
         <v>1</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N19" s="10" t="n">
         <v>2</v>
@@ -1805,7 +1799,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>2</v>
@@ -1817,10 +1811,10 @@
         <v>16</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H20" s="8" t="n">
         <v>4</v>
@@ -1829,16 +1823,16 @@
         <v>19</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="N20" s="10" t="n">
         <v>2</v>
@@ -1849,19 +1843,19 @@
         <v>21</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>2</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>18</v>
@@ -1873,7 +1867,7 @@
         <v>19</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K21" s="9" t="s">
         <v>19</v>
@@ -1882,7 +1876,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N21" s="10" t="n">
         <v>10</v>
@@ -1893,7 +1887,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>2</v>
@@ -1905,10 +1899,10 @@
         <v>16</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>7</v>
@@ -1920,13 +1914,13 @@
         <v>1</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>3</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N22" s="10" t="n">
         <v>3</v>
@@ -1949,10 +1943,10 @@
         <v>16</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="H23" s="8" t="n">
         <v>8</v>
@@ -1964,13 +1958,13 @@
         <v>1</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>3</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="N23" s="10" t="n">
         <v>3</v>
@@ -1993,16 +1987,16 @@
         <v>16</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H24" s="8" t="n">
         <v>6</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J24" s="8" t="n">
         <v>3</v>
@@ -2014,7 +2008,7 @@
         <v>3</v>
       </c>
       <c r="M24" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N24" s="10" t="n">
         <v>3</v>
@@ -2037,16 +2031,16 @@
         <v>16</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>8</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J25" s="8" t="n">
         <v>2</v>
@@ -2081,10 +2075,10 @@
         <v>16</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H26" s="8" t="n">
         <v>10</v>
@@ -2102,7 +2096,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="N26" s="10" t="n">
         <v>3</v>
@@ -2125,16 +2119,16 @@
         <v>16</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="H27" s="8" t="n">
         <v>10</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J27" s="8" t="n">
         <v>3</v>
@@ -2152,97 +2146,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="H28" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="J28" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="K28" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="L28" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="N28" s="10" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="n">
-        <v>29</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="H29" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="I29" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="J29" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="K29" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="L29" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="M29" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="N29" s="10" t="n">
-        <v>30</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G29" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G27" type="list">
       <formula1>INDIRECT("RarityData")</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2301,25 +2207,25 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="12" t="s">
         <v>77</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="M1" s="12" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2330,13 +2236,13 @@
         <v>20</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>17</v>
@@ -2369,13 +2275,13 @@
         <v>22</v>
       </c>
       <c r="C3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>17</v>
@@ -2408,13 +2314,13 @@
         <v>24</v>
       </c>
       <c r="C4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>17</v>
@@ -2447,13 +2353,13 @@
         <v>26</v>
       </c>
       <c r="C5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>17</v>
@@ -2486,13 +2392,13 @@
         <v>28</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>17</v>
@@ -2525,13 +2431,13 @@
         <v>30</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>17</v>
@@ -2564,13 +2470,13 @@
         <v>32</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>17</v>
@@ -2600,29 +2506,29 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="F9" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>10</v>
@@ -2642,13 +2548,13 @@
         <v>36</v>
       </c>
       <c r="C10" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>17</v>
@@ -2678,19 +2584,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="F11" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" s="7" t="n">
@@ -2720,13 +2626,13 @@
         <v>34</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>17</v>
@@ -2756,29 +2662,29 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="F13" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>10</v>
@@ -2795,19 +2701,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="F14" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7" t="n">
@@ -2834,19 +2740,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="F15" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="7" t="n">
@@ -2876,16 +2782,16 @@
         <v>68</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="F16" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7" t="n">
@@ -2949,10 +2855,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2965,34 +2871,34 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -3032,12 +2938,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
multiple balance adjustments (dragon buffs)
</commit_message>
<xml_diff>
--- a/Assets/Data/Data.xlsx
+++ b/Assets/Data/Data.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="106">
   <si>
     <t xml:space="preserve">Num Code</t>
   </si>
@@ -68,10 +68,10 @@
   </si>
   <si>
     <t xml:space="preserve">input=population:4;
-output=knight:4;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">flechery</t>
+output=knight:4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fletchery</t>
   </si>
   <si>
     <t xml:space="preserve">input=population:4;
@@ -130,7 +130,7 @@
 output=gunner:1</t>
   </si>
   <si>
-    <t xml:space="preserve">gem-transmutator</t>
+    <t xml:space="preserve">gem-transmutor</t>
   </si>
   <si>
     <t xml:space="preserve">Magic</t>
@@ -171,6 +171,51 @@
   </si>
   <si>
     <t xml:space="preserve">Peasantry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input=population:1;
+output=gem-income:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dragon-rider-roost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uncommon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input=dragon:1;
+output=dragon-rider:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">farm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input=population:1;
+output=pop-growth:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold-mine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input=population:1;
+output=gold:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">granary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input=population:1;
+output=pop-growth:2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trading-post</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input=population:1;
+output=gold:2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hunters-lodge</t>
   </si>
   <si>
     <r>
@@ -181,8 +226,8 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">input=population:1;
-output=</t>
+      <t xml:space="preserve">input=population:5;
+output=hunter</t>
     </r>
     <r>
       <rPr>
@@ -191,66 +236,8 @@
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">gem-income</t>
+      <t xml:space="preserve">:5|pop-growth:1</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">:1</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">dragon-rider-roost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uncommon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">input=dragon:1;
-output=dragon-rider:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">farm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">input=population:1;
-output=pop-growth:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold-mine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">input=population:1;
-output=gold:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">granary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">input=population:1;
-output=pop-growth:2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">trading-post</t>
-  </si>
-  <si>
-    <t xml:space="preserve">input=population:1;
-output=gold:2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hunters-lodge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">this is a long sentence. I am testing if this breaks. We will see</t>
-  </si>
-  <si>
-    <t xml:space="preserve">input=population:5;
-output=hunter:5|pop-growth:1</t>
   </si>
   <si>
     <t xml:space="preserve">mill</t>
@@ -284,36 +271,8 @@
     <t xml:space="preserve">crystal-refinery</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">input=population:2;
-output=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">gem-income</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">:3</t>
-    </r>
+    <t xml:space="preserve">input=population:2;
+output=gem-income:3</t>
   </si>
   <si>
     <t xml:space="preserve">mage-university</t>
@@ -1845,7 +1804,7 @@
         <v>2</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>11</v>
@@ -1860,7 +1819,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J21" s="8"/>
       <c r="K21" s="10"/>
@@ -1873,7 +1832,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>2</v>
@@ -1894,7 +1853,7 @@
         <v>7</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J22" s="8"/>
       <c r="K22" s="10"/>
@@ -1907,7 +1866,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>2</v>
@@ -1928,7 +1887,7 @@
         <v>8</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J23" s="8"/>
       <c r="K23" s="10"/>
@@ -1941,7 +1900,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>2</v>
@@ -1962,7 +1921,7 @@
         <v>6</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J24" s="8"/>
       <c r="K24" s="10"/>
@@ -1975,7 +1934,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>2</v>
@@ -1996,7 +1955,7 @@
         <v>8</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J25" s="8"/>
       <c r="K25" s="10"/>
@@ -2009,7 +1968,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>2</v>
@@ -2030,7 +1989,7 @@
         <v>10</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J26" s="8"/>
       <c r="K26" s="10"/>
@@ -2043,7 +2002,7 @@
         <v>27</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>2</v>
@@ -2064,7 +2023,7 @@
         <v>10</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J27" s="8"/>
       <c r="K27" s="10"/>
@@ -2120,8 +2079,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="12.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="12.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="12.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="12.8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2144,28 +2103,28 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2173,16 +2132,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>12</v>
@@ -2206,25 +2165,25 @@
         <v>2</v>
       </c>
       <c r="M2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="N2" s="14"/>
+    </row>
+    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="N2" s="14"/>
-    </row>
-    <row r="3" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>85</v>
-      </c>
       <c r="C3" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>12</v>
@@ -2248,10 +2207,10 @@
         <v>1</v>
       </c>
       <c r="M3" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="N3" s="15" t="s">
         <v>86</v>
-      </c>
-      <c r="N3" s="15" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2259,16 +2218,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C4" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>12</v>
@@ -2292,7 +2251,7 @@
         <v>1.5</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N4" s="14"/>
     </row>
@@ -2301,16 +2260,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C5" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>12</v>
@@ -2334,7 +2293,7 @@
         <v>3</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N5" s="15"/>
     </row>
@@ -2343,16 +2302,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>12</v>
@@ -2376,7 +2335,7 @@
         <v>0.2</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N6" s="14"/>
     </row>
@@ -2385,16 +2344,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>12</v>
@@ -2418,7 +2377,7 @@
         <v>6</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N7" s="15"/>
     </row>
@@ -2427,16 +2386,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>12</v>
@@ -2460,7 +2419,7 @@
         <v>1.5</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N8" s="14"/>
     </row>
@@ -2469,16 +2428,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>39</v>
@@ -2502,25 +2461,25 @@
         <v>4</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N9" s="15"/>
     </row>
-    <row r="10" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C10" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>12</v>
@@ -2544,10 +2503,10 @@
         <v>0.5</v>
       </c>
       <c r="M10" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="N10" s="14" t="s">
         <v>86</v>
-      </c>
-      <c r="N10" s="14" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2555,16 +2514,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="E11" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>44</v>
@@ -2588,7 +2547,7 @@
         <v>1</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N11" s="15"/>
     </row>
@@ -2597,16 +2556,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="E12" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>28</v>
@@ -2630,10 +2589,10 @@
         <v>1</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N12" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2641,16 +2600,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>39</v>
@@ -2674,25 +2633,25 @@
         <v>4</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N13" s="15"/>
     </row>
-    <row r="14" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>33</v>
@@ -2716,27 +2675,27 @@
         <v>1</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N14" s="14" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="E15" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>44</v>
@@ -2760,27 +2719,27 @@
         <v>1</v>
       </c>
       <c r="M15" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="N15" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="N15" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>33</v>
@@ -2804,10 +2763,10 @@
         <v>1</v>
       </c>
       <c r="M16" s="16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N16" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2846,50 +2805,50 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>